<commit_message>
fix(viewer): refresh authored sample after column coalescing
</commit_message>
<xml_diff>
--- a/viewer/samples/operations-report.xlsx
+++ b/viewer/samples/operations-report.xlsx
@@ -224,8 +224,7 @@
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="3" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -393,9 +392,7 @@
   </sheetPr>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="2" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>